<commit_message>
fix: resolve ImportError and fix G2B data retrieval logic
</commit_message>
<xml_diff>
--- a/샘플데이터/사업체정보_표준양식_샘플_사업자번호.xlsx
+++ b/샘플데이터/사업체정보_표준양식_샘플_사업자번호.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\app\1.보고서 분석기\샘플데이터\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF27955E-AAFE-4F3F-A078-F8F39C2F38E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4212F2E0-6508-42C3-B89E-83A24B42F917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28920" yWindow="-16380" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="사업체목록" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="110">
   <si>
     <t>사업자등록번호</t>
   </si>
@@ -535,6 +535,18 @@
   <si>
     <t xml:space="preserve">경기 용인시 기흥구 마북로 207                                                                                                     </t>
   </si>
+  <si>
+    <t>메트릭스</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>나윤정, 조일상</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울특별시 서초구 강남대로6길 11</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -632,13 +644,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1034,7 +1049,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D5661"/>
+  <dimension ref="A1:D5662"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.625" customWidth="1"/>
@@ -1058,382 +1073,391 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3" t="s">
-        <v>25</v>
+      <c r="A2" s="4">
+        <v>3248801602</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>51</v>
+      <c r="B2" s="4" t="s">
+        <v>107</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>76</v>
+      <c r="C2" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
       <c r="B3" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
       <c r="B4" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
       <c r="B5" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
       <c r="B7" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B10" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B11" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B12" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B13" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B14" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C14" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D14" s="3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B15" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B17" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C17" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D17" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B18" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C18" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D18" s="3" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B19" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D19" s="3" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B20" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C20" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B21" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C21" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D21" s="3" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B22" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C22" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B23" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C23" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B24" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C24" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D24" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B25" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C25" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C26" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D26" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B27" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C27" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D27" s="3" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="3" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B28" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C28" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D28" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B29" s="3" t="s">
         <v>102</v>
-      </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B29" s="3" t="s">
-        <v>105</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B30" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C30" s="2"/>
+      <c r="D30" s="3" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B31" s="2"/>
@@ -29590,19 +29614,24 @@
       <c r="C5661" s="2"/>
       <c r="D5661" s="2"/>
     </row>
+    <row r="5662" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B5662" s="2"/>
+      <c r="C5662" s="2"/>
+      <c r="D5662" s="2"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="B2:B27">
+  <conditionalFormatting sqref="B3:B28">
     <cfRule type="duplicateValues" dxfId="8" priority="7"/>
     <cfRule type="duplicateValues" dxfId="7" priority="8"/>
     <cfRule type="duplicateValues" dxfId="6" priority="9"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B28">
+  <conditionalFormatting sqref="B29">
     <cfRule type="duplicateValues" dxfId="5" priority="4"/>
     <cfRule type="duplicateValues" dxfId="4" priority="5"/>
     <cfRule type="duplicateValues" dxfId="3" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B29">
+  <conditionalFormatting sqref="B30">
     <cfRule type="duplicateValues" dxfId="2" priority="1"/>
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
     <cfRule type="duplicateValues" dxfId="0" priority="3"/>

</xml_diff>